<commit_message>
New rubric for lab 5B
</commit_message>
<xml_diff>
--- a/Labs/Lab4/Assignment4Rubric.xlsx
+++ b/Labs/Lab4/Assignment4Rubric.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/DataCard/Repos/CS246-CourseMaterials/Labs/Lab4/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/birdb/Projects/CS246-CourseMaterials/Labs/Lab4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76CEFCF-422E-7348-95A5-5F695A9920CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F8B90B-CCD3-D64C-955B-C1C47F065CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9960" yWindow="600" windowWidth="13920" windowHeight="14640" activeTab="1" xr2:uid="{2ED55EEA-81A7-FF44-BCE3-68AB9ADB8259}"/>
+    <workbookView xWindow="-27400" yWindow="500" windowWidth="18900" windowHeight="20240" activeTab="1" xr2:uid="{2ED55EEA-81A7-FF44-BCE3-68AB9ADB8259}"/>
   </bookViews>
   <sheets>
     <sheet name="Rubric" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="23">
   <si>
     <t>Requirements</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>Correctly done</t>
+  </si>
+  <si>
+    <t>Your OO design looks good and the UML diagram is correctly done.</t>
   </si>
 </sst>
 </file>
@@ -187,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -206,6 +209,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -661,7 +670,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8EF6DB9-5046-F545-B378-AB8AF91CAAF1}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="28.33203125" customWidth="1"/>
@@ -669,21 +678,22 @@
     <col min="3" max="3" width="7" customWidth="1"/>
     <col min="4" max="4" width="1.1640625" customWidth="1"/>
     <col min="5" max="5" width="22.33203125" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="20" customHeight="1">
+    <row r="3" spans="1:6" ht="20" customHeight="1">
       <c r="A3" s="10" t="s">
         <v>17</v>
       </c>
@@ -692,156 +702,179 @@
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:6" ht="20" customHeight="1">
+      <c r="A4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="7" t="s">
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B6" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="17">
-      <c r="A6" s="4" t="s">
+      <c r="E6" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="17">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2">
-        <v>15</v>
-      </c>
-      <c r="E6" s="9" t="s">
+      <c r="B7" s="2">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2">
+        <v>15</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="17">
-      <c r="A7" s="4" t="s">
+      <c r="F7" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="17">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2">
-        <v>15</v>
-      </c>
-      <c r="C7" s="2">
-        <v>15</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="17">
-      <c r="A8" s="4" t="s">
+      <c r="B8" s="2">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2">
+        <v>15</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="17">
+      <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2">
-        <v>20</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="B9" s="2">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2">
+        <v>20</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="6" t="s">
+      <c r="F9" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" spans="1:5" ht="17">
-      <c r="A10" s="4" t="s">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="17">
+      <c r="A11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2">
-        <v>15</v>
-      </c>
-      <c r="C10" s="2">
-        <v>15</v>
-      </c>
-      <c r="E10" s="9" t="s">
+      <c r="B11" s="2">
+        <v>15</v>
+      </c>
+      <c r="C11" s="2">
+        <v>15</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="17">
-      <c r="A11" s="4" t="s">
+      <c r="F11" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="17">
+      <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="2">
-        <v>20</v>
-      </c>
-      <c r="C11" s="2">
-        <v>20</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="5" customFormat="1" ht="17">
-      <c r="A12" s="4" t="s">
+      <c r="B12" s="2">
+        <v>20</v>
+      </c>
+      <c r="C12" s="2">
+        <v>20</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="5" customFormat="1" ht="17">
+      <c r="A13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="2">
-        <v>15</v>
-      </c>
-      <c r="C12" s="2">
-        <v>15</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="4" t="s">
+      <c r="B13" s="2">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2">
+        <v>15</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="2">
-        <f>SUM(B6:B12)</f>
+      <c r="B14" s="2">
+        <f>SUM(B7:B13)</f>
         <v>100</v>
       </c>
-      <c r="C13" s="2">
-        <f>SUM(C6:C12)</f>
+      <c r="C14" s="2">
+        <f>SUM(C7:C13)</f>
         <v>100</v>
       </c>
-      <c r="E13" s="9"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="4"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="4" t="s">
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="4"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="4" t="s">
+      <c r="B16" s="1"/>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="4"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
     </row>
@@ -850,14 +883,20 @@
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
     </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
+    <row r="19" spans="1:3">
+      <c r="A19" s="4"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A4:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>